<commit_message>
Corrige classificação Tipo: Comum (outro Fund II) para professores como AMu com turmas 7C
Co-authored-by: cbrener89052 <cbrener89052@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/professores_comuns_reuniao_C_2026.xlsx
+++ b/professores_comuns_reuniao_C_2026.xlsx
@@ -29,10 +29,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0E0E3"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -101,6 +106,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -468,22 +476,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -496,12 +507,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TL Fund II (6C+7C)</t>
+          <t>TL bloco Fund II (6C+7C)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TL EM (9C+10C)</t>
+          <t>TL bloco EM (9C+10C)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -516,12 +527,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Turmas Fund II (6C+7C)</t>
+          <t>Turmas bloco Fund II (6C+7C)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Disciplinas Fund II</t>
+          <t>Disciplinas bloco Fund II</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -532,6 +543,21 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Disciplinas EM</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Outras turmas Fund II (C)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Disciplinas outro Fund II</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Observação</t>
         </is>
       </c>
     </row>
@@ -582,6 +608,21 @@
           <t>esp</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -630,6 +671,21 @@
           <t>his</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -678,6 +734,21 @@
           <t>appor</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -690,10 +761,8 @@
           <t>ANZI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C5" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>4</v>
@@ -728,11 +797,26 @@
           <t>proj port cult</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -740,10 +824,8 @@
           <t>APa</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>16</v>
@@ -778,11 +860,26 @@
           <t>ing, ingT, proj port soc</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 5C1, 5C2, 5C3 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -790,10 +887,8 @@
           <t>Ale</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>8</v>
@@ -828,6 +923,21 @@
           <t>bio, proj port amb</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>cie</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 8C1, 8C2 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -876,11 +986,26 @@
           <t>pred</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>appor, pgram</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -888,10 +1013,8 @@
           <t>BrSa</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>16</v>
@@ -926,6 +1049,21 @@
           <t>mat</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>apmat</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 8C1, 8C2 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -938,10 +1076,8 @@
           <t>CAl</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>4</v>
@@ -976,6 +1112,21 @@
           <t>qui</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -988,10 +1139,8 @@
           <t>Car</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>4</v>
@@ -1026,6 +1175,21 @@
           <t>GL</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1074,6 +1238,21 @@
           <t>DaF, GL, ap DaF</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>DaF</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1122,6 +1301,21 @@
           <t>mus</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>mus</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1170,6 +1364,21 @@
           <t>art</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>art</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1218,11 +1427,26 @@
           <t>ese</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>ese</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1230,10 +1454,8 @@
           <t>EFr</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C16" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>32</v>
@@ -1268,6 +1490,21 @@
           <t>DaF, GL</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>GL</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 8C1, 8C2 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1316,6 +1553,21 @@
           <t>apmat, mat</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>8C1</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1328,10 +1580,8 @@
           <t>Fab</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C18" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>2</v>
@@ -1366,11 +1616,26 @@
           <t>qui</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1378,10 +1643,8 @@
           <t>Jana</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>4</v>
@@ -1416,6 +1679,21 @@
           <t>p</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>pgram</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 8C1, 8C2 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1428,10 +1706,8 @@
           <t>Joa</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C20" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>10</v>
@@ -1466,6 +1742,21 @@
           <t>artTh, elet arte sm</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1514,6 +1805,21 @@
           <t>his</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>ese, eso</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1526,10 +1832,8 @@
           <t>Kle</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C22" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>2</v>
@@ -1564,6 +1868,21 @@
           <t>soc</t>
         </is>
       </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1612,6 +1931,21 @@
           <t>DaF, GL</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1624,10 +1958,8 @@
           <t>LAn</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C24" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>4</v>
@@ -1662,6 +1994,21 @@
           <t>elet hist cult filo, fil</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1710,6 +2057,21 @@
           <t>esp</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1722,10 +2084,8 @@
           <t>Lza</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>6</v>
@@ -1760,6 +2120,21 @@
           <t>bio</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1808,6 +2183,21 @@
           <t>plit</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1820,10 +2210,8 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C28" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>4</v>
@@ -1858,11 +2246,26 @@
           <t>geo</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1870,10 +2273,8 @@
           <t>Mlo</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C29" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>6</v>
@@ -1908,6 +2309,21 @@
           <t>finan, geo</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 8C1, 8C2 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1956,6 +2372,21 @@
           <t>ingT</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1968,10 +2399,8 @@
           <t>Raf</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>6</v>
@@ -2006,6 +2435,21 @@
           <t>pred</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2054,6 +2498,21 @@
           <t>esp</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2102,6 +2561,21 @@
           <t>DaF, ap DaF</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2114,10 +2588,8 @@
           <t>SJu</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C34" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>6</v>
@@ -2152,11 +2624,26 @@
           <t>proj port tec, tec</t>
         </is>
       </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2164,10 +2651,8 @@
           <t>SMo</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C35" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>2</v>
@@ -2202,6 +2687,21 @@
           <t>p</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 5C1, 5C2, 5C3 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2250,6 +2750,21 @@
           <t>tec</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>tec</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2262,10 +2777,8 @@
           <t>VSi</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C37" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>8</v>
@@ -2300,6 +2813,21 @@
           <t>elet mod 3D, fis</t>
         </is>
       </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2348,6 +2876,21 @@
           <t>ingT</t>
         </is>
       </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2394,6 +2937,21 @@
       <c r="J39" s="2" t="inlineStr">
         <is>
           <t>ing</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>5C2</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2408,22 +2966,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -2436,12 +2997,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TL Fund II (5C+8C)</t>
+          <t>TL bloco Fund II (5C+8C)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TL EM (11C+12C)</t>
+          <t>TL bloco EM (11C+12C)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2456,12 +3017,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Turmas Fund II (5C+8C)</t>
+          <t>Turmas bloco Fund II (5C+8C)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Disciplinas Fund II</t>
+          <t>Disciplinas bloco Fund II</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -2472,6 +3033,21 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Disciplinas EM</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Outras turmas Fund II (C)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Disciplinas outro Fund II</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Observação</t>
         </is>
       </c>
     </row>
@@ -2522,6 +3098,21 @@
           <t>pred</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2570,11 +3161,26 @@
           <t>esp</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2582,10 +3188,8 @@
           <t>AMu</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>8</v>
@@ -2620,6 +3224,21 @@
           <t>plit, pred</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 7C1, 7C2, 7C3 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2668,6 +3287,21 @@
           <t>apr bio, bio</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2716,6 +3350,21 @@
           <t>ing</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2728,10 +3377,8 @@
           <t>Bre</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>12</v>
@@ -2766,6 +3413,21 @@
           <t>apr mat, mat</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -2778,10 +3440,8 @@
           <t>CAl</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>10</v>
@@ -2816,6 +3476,21 @@
           <t>apr qui, qui</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -2828,10 +3503,8 @@
           <t>CBu</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>28</v>
@@ -2866,6 +3539,21 @@
           <t>DaF, GL</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -2878,10 +3566,8 @@
           <t>Cadu</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>18</v>
@@ -2916,6 +3602,21 @@
           <t>apr fís, fis</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2964,6 +3665,21 @@
           <t>mat</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>7C3</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3012,11 +3728,26 @@
           <t>mus</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>mus</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -3024,10 +3755,8 @@
           <t>Deb</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C13" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>8</v>
@@ -3062,6 +3791,21 @@
           <t>plit</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>pgram</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 6C1, 6C2, 7C1, 7C2, 7C3 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3110,6 +3854,21 @@
           <t>art</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>art</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3158,6 +3917,21 @@
           <t>DaF, GL</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -3170,10 +3944,8 @@
           <t>Fab</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C16" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>8</v>
@@ -3208,6 +3980,21 @@
           <t>apr qui, qui</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3256,11 +4043,26 @@
           <t>ing</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3268,10 +4070,8 @@
           <t>JCa</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C18" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>4</v>
@@ -3306,6 +4106,21 @@
           <t>apr geo</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 6C1, 6C2, 6C3, 7C1, 7C2, 7C3 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -3318,10 +4133,8 @@
           <t>JJ</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>8</v>
@@ -3356,6 +4169,21 @@
           <t>mat</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -3368,10 +4196,8 @@
           <t>Joa</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C20" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>8</v>
@@ -3406,6 +4232,21 @@
           <t>artTh</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -3418,10 +4259,8 @@
           <t>Kle</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C21" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>4</v>
@@ -3456,6 +4295,21 @@
           <t>soc</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3504,6 +4358,21 @@
           <t>DaF, GL</t>
         </is>
       </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>7C3</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>DaF</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -3516,10 +4385,8 @@
           <t>LAn</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C23" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>4</v>
@@ -3554,6 +4421,21 @@
           <t>fil</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -3566,10 +4448,8 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C24" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>14</v>
@@ -3604,6 +4484,21 @@
           <t>apr geo, geo</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3652,6 +4547,21 @@
           <t>ing</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -3664,10 +4574,8 @@
           <t>Raf</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>2</v>
@@ -3702,6 +4610,21 @@
           <t>p</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3750,11 +4673,26 @@
           <t>esp</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Só EM</t>
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Comum (outro Fund II)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3762,10 +4700,8 @@
           <t>SGa</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C28" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>14</v>
@@ -3800,6 +4736,21 @@
           <t>DaF, GL</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Leciona também em 7C1, 7C2, 7C3 — ver outra aba</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3812,10 +4763,8 @@
           <t>Ver</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C29" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>6</v>
@@ -3850,6 +4799,21 @@
           <t>his</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -3862,10 +4826,8 @@
           <t>Wag</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>14</v>
@@ -3898,6 +4860,21 @@
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t>apr his, his</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona aba Carga EFII vs EM com TL total por professor no ramo C
Co-authored-by: cbrener89052 <cbrener89052@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/professores_comuns_reuniao_C_2026.xlsx
+++ b/professores_comuns_reuniao_C_2026.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="6C-7C vs 9C-10C" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="5C-8C vs 11C-12C" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Carga EFII vs EM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="6C-7C vs 9C-10C" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="5C-8C vs 11C-12C" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -46,22 +47,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE5CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D0E0E3"/>
+        <fgColor rgb="00E8E8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -106,9 +102,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -476,6 +469,2916 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>TL EFII (5C-8C)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TL EM (9C-12C)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Maior carga horária</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Segmentos (C)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Turmas EFII</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Turmas EM</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Disciplinas EFII</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Disciplinas EM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EFr</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>GL</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>LUR</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL, ap DaF novo</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Tha</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Velo</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>aping, ingT</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>cie</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>apr bio, bio, proj port amb</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Bea</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>11C1</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>ing</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CBu</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Krk</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SGa</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL, ap DaF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C2</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Jad</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 6C3, 7C1</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LBa</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>apmat, mat</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ADo</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Caro</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>DaF</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL, ap DaF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Luc</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Ron</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 7C1, 7C2</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Vir</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>5C2, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>10C2</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>ing</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>MMi</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL, ap DaF</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Cadu</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>apr fís, fis</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>DCo</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>esp</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>JOL</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>DaF, GL</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Joa</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>artTh, elet arte sm</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>apr geo, geo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>PaH</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>11C2, 12C1, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>ing, ingT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Raq</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>cie</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>APa</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>ing, ingT, proj port soc</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>BrSa</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>apmat</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>DeBra</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>mus</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>mus</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Dei</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>art</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>art</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>CAl</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>apr qui, qui</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Wag</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>apr his, his</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ALu</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>his</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>his</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Bre</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>apr mat, mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>JCa</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>apr geo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>JuLa</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>ese, eso</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>his</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>MFo</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>appor, pred</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>plit</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>BPad</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C3</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>appor, pgram</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Tac</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3, 6C1, 6C2, 6C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>10C2, 9C2</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>tec</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>tec</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>AMu</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>appor, plit, pred</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>ClaMe</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>7C3, 8C2</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Deb</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>pgram</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>plit</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>FBri</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>6C3, 8C1</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>apmat, mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Fab</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>apr qui, qui</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>MSM</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>5C3, 7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>appor, ingT</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>SMo</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>JJ</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>LAn</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>elet hist cult filo, fil</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Raf</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>p, pred</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>VSi</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>elet mod 3D, fis</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>ACo</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>pred</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Kle</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 11C1, 11C2, 12C1, 12C2</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>soc</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Lza</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>bio</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Mlo</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>finan, geo</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>RSE</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>art</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>SJu</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2, 9C1</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>proj port tec, tec</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>11C1, 11C2</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>his</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>DiS</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3, 8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>ese</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>ese</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Isb</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>5C1</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>12C2</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>ingT</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>ing</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>ABa</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>his</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>ANZI</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>proj port cult</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>10C1, 10C2</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>GL</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Jana</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Empate</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>EFII + EM</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>8C1, 8C2</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>9C1, 9C2</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>pgram</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Dla</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>6C1, 6C2, 6C3</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>ap DaF</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>MoPa</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>5C1, 5C2, 5C3</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>ap DaF</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Sil</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>EFII</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>7C1, 7C2, 7C3</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>ap DaF</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -491,10 +3394,10 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="27" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -578,7 +3481,7 @@
       <c r="D2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -641,7 +3544,7 @@
       <c r="D3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -704,7 +3607,7 @@
       <c r="D4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -751,7 +3654,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -767,7 +3670,7 @@
       <c r="D5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -814,7 +3717,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -830,7 +3733,7 @@
       <c r="D6" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -877,7 +3780,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -893,7 +3796,7 @@
       <c r="D7" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -956,7 +3859,7 @@
       <c r="D8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1003,7 +3906,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -1019,7 +3922,7 @@
       <c r="D9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1066,7 +3969,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -1082,7 +3985,7 @@
       <c r="D10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1129,7 +4032,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -1145,7 +4048,7 @@
       <c r="D11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1208,7 +4111,7 @@
       <c r="D12" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1271,7 +4174,7 @@
       <c r="D13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1334,7 +4237,7 @@
       <c r="D14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1397,7 +4300,7 @@
       <c r="D15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -1444,7 +4347,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -1460,7 +4363,7 @@
       <c r="D16" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1523,7 +4426,7 @@
       <c r="D17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1570,7 +4473,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -1586,7 +4489,7 @@
       <c r="D18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1633,7 +4536,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -1649,7 +4552,7 @@
       <c r="D19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1696,7 +4599,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -1712,7 +4615,7 @@
       <c r="D20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1775,7 +4678,7 @@
       <c r="D21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1822,7 +4725,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -1838,7 +4741,7 @@
       <c r="D22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1901,7 +4804,7 @@
       <c r="D23" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -1948,7 +4851,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -1964,7 +4867,7 @@
       <c r="D24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2027,7 +4930,7 @@
       <c r="D25" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2074,7 +4977,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -2090,7 +4993,7 @@
       <c r="D26" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2153,7 +5056,7 @@
       <c r="D27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2200,7 +5103,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -2216,7 +5119,7 @@
       <c r="D28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2263,7 +5166,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -2279,7 +5182,7 @@
       <c r="D29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2342,7 +5245,7 @@
       <c r="D30" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2389,7 +5292,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -2405,7 +5308,7 @@
       <c r="D31" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2468,7 +5371,7 @@
       <c r="D32" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2531,7 +5434,7 @@
       <c r="D33" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2578,7 +5481,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -2594,7 +5497,7 @@
       <c r="D34" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2641,7 +5544,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -2657,7 +5560,7 @@
       <c r="D35" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2720,7 +5623,7 @@
       <c r="D36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2767,7 +5670,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -2783,7 +5686,7 @@
       <c r="D37" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -2846,7 +5749,7 @@
       <c r="D38" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2909,7 +5812,7 @@
       <c r="D39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -2960,7 +5863,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2981,10 +5884,10 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -3068,7 +5971,7 @@
       <c r="D2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3131,7 +6034,7 @@
       <c r="D3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3178,7 +6081,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -3194,7 +6097,7 @@
       <c r="D4" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3257,7 +6160,7 @@
       <c r="D5" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3320,7 +6223,7 @@
       <c r="D6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -3367,7 +6270,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -3383,7 +6286,7 @@
       <c r="D7" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3430,7 +6333,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -3446,7 +6349,7 @@
       <c r="D8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3493,7 +6396,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -3509,7 +6412,7 @@
       <c r="D9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3556,7 +6459,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -3572,7 +6475,7 @@
       <c r="D10" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3635,7 +6538,7 @@
       <c r="D11" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3698,7 +6601,7 @@
       <c r="D12" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3745,7 +6648,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -3761,7 +6664,7 @@
       <c r="D13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3824,7 +6727,7 @@
       <c r="D14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3887,7 +6790,7 @@
       <c r="D15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -3934,7 +6837,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -3950,7 +6853,7 @@
       <c r="D16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4013,7 +6916,7 @@
       <c r="D17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -4060,7 +6963,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -4076,7 +6979,7 @@
       <c r="D18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4123,7 +7026,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4139,7 +7042,7 @@
       <c r="D19" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4186,7 +7089,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4202,7 +7105,7 @@
       <c r="D20" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4249,7 +7152,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4265,7 +7168,7 @@
       <c r="D21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4328,7 +7231,7 @@
       <c r="D22" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -4375,7 +7278,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4391,7 +7294,7 @@
       <c r="D23" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4438,7 +7341,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4454,7 +7357,7 @@
       <c r="D24" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4517,7 +7420,7 @@
       <c r="D25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -4564,7 +7467,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4580,7 +7483,7 @@
       <c r="D26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4643,7 +7546,7 @@
       <c r="D27" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>EFII</t>
         </is>
@@ -4690,7 +7593,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Comum (outro Fund II)</t>
         </is>
@@ -4706,7 +7609,7 @@
       <c r="D28" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4753,7 +7656,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4769,7 +7672,7 @@
       <c r="D29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
@@ -4816,7 +7719,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Só EM</t>
         </is>
@@ -4832,7 +7735,7 @@
       <c r="D30" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>EM</t>
         </is>

</xml_diff>